<commit_message>
Dapine v4.0 - 91 steps across 3 tests. Pivot, Try/Catch, Export SQL, Window. ALL PASSING.
</commit_message>
<xml_diff>
--- a/final_output.xlsx
+++ b/final_output.xlsx
@@ -59,9 +59,7 @@
   </cellStyleXfs>
   <cellXfs count="2">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="1" fillId="2" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center"/>
-    </xf>
+    <xf numFmtId="0" fontId="1" fillId="2" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
@@ -427,19 +425,20 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D4"/>
+  <dimension ref="A1:E3"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
-    <col width="10" customWidth="1" min="1" max="1"/>
+    <col width="6" customWidth="1" min="1" max="1"/>
     <col width="7" customWidth="1" min="2" max="2"/>
-    <col width="11" customWidth="1" min="3" max="3"/>
+    <col width="10" customWidth="1" min="3" max="3"/>
     <col width="10" customWidth="1" min="4" max="4"/>
+    <col width="10" customWidth="1" min="5" max="5"/>
   </cols>
   <sheetData>
     <row r="1">
       <c r="A1" s="1" t="inlineStr">
         <is>
-          <t>bedrooms</t>
+          <t>beds</t>
         </is>
       </c>
       <c r="B1" s="1" t="inlineStr">
@@ -449,55 +448,56 @@
       </c>
       <c r="C1" s="1" t="inlineStr">
         <is>
-          <t>avg_price</t>
+          <t>avg_cost</t>
         </is>
       </c>
       <c r="D1" s="1" t="inlineStr">
         <is>
           <t>cheapest</t>
+        </is>
+      </c>
+      <c r="E1" s="1" t="inlineStr">
+        <is>
+          <t>priciest</t>
         </is>
       </c>
     </row>
     <row r="2">
-      <c r="A2" t="n">
-        <v>4</v>
+      <c r="A2" t="inlineStr">
+        <is>
+          <t>5</t>
+        </is>
       </c>
       <c r="B2" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="C2" t="n">
-        <v>450000</v>
+        <v>575000</v>
       </c>
       <c r="D2" t="n">
-        <v>400000</v>
+        <v>550000</v>
+      </c>
+      <c r="E2" t="n">
+        <v>600000</v>
       </c>
     </row>
     <row r="3">
-      <c r="A3" t="n">
-        <v>3</v>
+      <c r="A3" t="inlineStr">
+        <is>
+          <t>4</t>
+        </is>
       </c>
       <c r="B3" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="C3" t="n">
-        <v>325000</v>
+        <v>500000</v>
       </c>
       <c r="D3" t="n">
-        <v>300000</v>
-      </c>
-    </row>
-    <row r="4">
-      <c r="A4" t="n">
-        <v>5</v>
-      </c>
-      <c r="B4" t="n">
-        <v>2</v>
-      </c>
-      <c r="C4" t="n">
-        <v>575000</v>
-      </c>
-      <c r="D4" t="n">
-        <v>550000</v>
+        <v>500000</v>
+      </c>
+      <c r="E3" t="n">
+        <v>500000</v>
       </c>
     </row>
   </sheetData>

</xml_diff>